<commit_message>
feat: update scheduler all module fix api http test
</commit_message>
<xml_diff>
--- a/documents/SmartMoney_Final.xlsx
+++ b/documents/SmartMoney_Final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ducph\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E90F22-9388-459D-A03C-10D65E84DABC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC92E2E3-D9E4-497F-9457-29A781DE50EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="202">
   <si>
     <t>🗂️  SMARTMONEY – PHÂN CÔNG CÔNG VIỆC  |  19/03/2026 → 23/04/2026</t>
   </si>
@@ -199,15 +199,9 @@
     <t xml:space="preserve">  ▸  Xây dựng UI/UX Mobile (Flutter/Dart) – Menu cho toàn giao diện mobile</t>
   </si>
   <si>
-    <t>tEvents, tBudgets</t>
-  </si>
-  <si>
     <t>Flutter 3.38.7, Dart SDK ≥3.10.7, Android SDK 30</t>
   </si>
   <si>
-    <t xml:space="preserve">  ▸  Tích hợp API từ 2 module backend (tEvents, tBudgets)</t>
-  </si>
-  <si>
     <t xml:space="preserve">  ▸  Biểu đồ thống kê chi tiêu (fl_chart 0.66.2)</t>
   </si>
   <si>
@@ -269,12 +263,6 @@
   </si>
   <si>
     <t>Duy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ▸  Tích hợp API từ 2 module backend (tWallets, tSavingGoals)</t>
-  </si>
-  <si>
-    <t>tWallets, tSavingGoals</t>
   </si>
   <si>
     <t>5</t>
@@ -615,6 +603,48 @@
   </si>
   <si>
     <t>https://github.com/ducphatdeveloper/SmartMoney_ProjectHK4_Group03</t>
+  </si>
+  <si>
+    <t>tEvents, tSavingGoals</t>
+  </si>
+  <si>
+    <t>tWallets, tBudgets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ▸  Tích hợp API từ 2 module backend (tWallets, tBudgets)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ▸  Tích hợp API từ 2 module backend (tEvents, tSavingGoals)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ▸  Tính năng thông báo trong flutter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ▸  Register</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ▸  Login</t>
+  </si>
+  <si>
+    <t>🔄 80%</t>
+  </si>
+  <si>
+    <t>🔄 70%</t>
+  </si>
+  <si>
+    <t>đang làm document review 3 ( wallet xong budget 4/5/2026 bắt đầu làm )</t>
+  </si>
+  <si>
+    <t>Hỗ trợ nhóm merge code fix lỗi, hướng dẫn,….</t>
+  </si>
+  <si>
+    <t>SPRING BOOT SERVER API + Flutter</t>
+  </si>
+  <si>
+    <t>đang fix lại admin, chuẩn bị bổ sung cột tcontacts 4/5/2026</t>
+  </si>
+  <si>
+    <t>Phụ dịch doc sang tiếng việt 4/4/2026</t>
   </si>
 </sst>
 </file>
@@ -624,7 +654,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -805,8 +835,15 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="32">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -993,8 +1030,55 @@
         <bgColor rgb="FFEAF2FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFEAECEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FF1E8449"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFEAFAF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFEAF2FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFF5EAF9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFF0FAF4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFFDEBD0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1030,12 +1114,86 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC8C8C8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC8C8C8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC8C8C8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC8C8C8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFC8C8C8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFC8C8C8"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFC8C8C8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFC8C8C8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFC8C8C8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFC8C8C8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFC8C8C8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFC8C8C8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="26" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1098,12 +1256,6 @@
     <xf numFmtId="0" fontId="8" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1155,29 +1307,100 @@
     <xf numFmtId="0" fontId="21" fillId="31" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="28" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="23" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1185,21 +1408,48 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="39" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Accent2" xfId="2" builtinId="33"/>
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
     <cellStyle name="Siêu kết nối" xfId="1" builtinId="8"/>
   </cellStyles>
@@ -1463,7 +1713,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1475,37 +1725,38 @@
     <col min="7" max="8" width="13" customWidth="1"/>
     <col min="9" max="9" width="8" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="39.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+    <row r="1" spans="1:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="72" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-    </row>
-    <row r="2" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+    </row>
+    <row r="2" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
-    </row>
-    <row r="3" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+    </row>
+    <row r="3" spans="1:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1519,7 +1770,7 @@
         <v>5</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>6</v>
@@ -1528,7 +1779,7 @@
         <v>7</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>8</v>
@@ -1537,11 +1788,11 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="s">
+    <row r="4" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="74" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -1569,9 +1820,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="51"/>
-      <c r="B5" s="51"/>
+    <row r="5" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="78"/>
+      <c r="B5" s="75"/>
       <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
@@ -1598,9 +1849,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="51"/>
-      <c r="B6" s="51"/>
+    <row r="6" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="78"/>
+      <c r="B6" s="75"/>
       <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
@@ -1626,9 +1877,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="51"/>
-      <c r="B7" s="51"/>
+    <row r="7" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="78"/>
+      <c r="B7" s="75"/>
       <c r="C7" s="2" t="s">
         <v>12</v>
       </c>
@@ -1639,7 +1890,7 @@
         <v>26</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="G7" s="8">
         <v>46100</v>
@@ -1655,9 +1906,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="51"/>
-      <c r="B8" s="51"/>
+    <row r="8" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="78"/>
+      <c r="B8" s="75"/>
       <c r="C8" s="2" t="s">
         <v>12</v>
       </c>
@@ -1683,9 +1934,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="51"/>
-      <c r="B9" s="51"/>
+    <row r="9" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="78"/>
+      <c r="B9" s="75"/>
       <c r="C9" s="13" t="s">
         <v>31</v>
       </c>
@@ -1712,9 +1963,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="51"/>
-      <c r="B10" s="51"/>
+    <row r="10" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="78"/>
+      <c r="B10" s="75"/>
       <c r="C10" s="13" t="s">
         <v>31</v>
       </c>
@@ -1731,71 +1982,92 @@
         <v>46100</v>
       </c>
       <c r="H10" s="9">
-        <v>46105</v>
+        <v>46117</v>
       </c>
       <c r="I10" s="10">
         <f>H10-G10</f>
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-    </row>
-    <row r="12" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53" t="s">
+        <v>196</v>
+      </c>
+      <c r="K10" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="78"/>
+      <c r="B11" s="75"/>
+      <c r="C11" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="G11" s="8">
+        <v>46106</v>
+      </c>
+      <c r="H11" s="9">
+        <v>46107</v>
+      </c>
+      <c r="I11" s="10">
+        <f>H11-G11</f>
+        <v>1</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="79"/>
+      <c r="B12" s="76"/>
+      <c r="C12" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" s="8">
+        <v>46109</v>
+      </c>
+      <c r="H12" s="9">
+        <v>46111</v>
+      </c>
+      <c r="I12" s="10">
+        <f>H12-G12</f>
+        <v>2</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="54" t="s">
+      <c r="B13" s="80" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="G12" s="8">
-        <v>46100</v>
-      </c>
-      <c r="H12" s="9">
-        <v>46100</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J12" s="7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="53"/>
-      <c r="B13" s="53"/>
       <c r="C13" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>40</v>
@@ -1813,17 +2085,17 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="53"/>
-      <c r="B14" s="53"/>
+    <row r="14" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="84"/>
+      <c r="B14" s="81"/>
       <c r="C14" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>40</v>
@@ -1841,17 +2113,17 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="53"/>
-      <c r="B15" s="53"/>
+    <row r="15" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="84"/>
+      <c r="B15" s="81"/>
       <c r="C15" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>40</v>
@@ -1869,20 +2141,20 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="53"/>
-      <c r="B16" s="53"/>
+    <row r="16" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="84"/>
+      <c r="B16" s="81"/>
       <c r="C16" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="G16" s="8">
         <v>46100</v>
@@ -1897,20 +2169,20 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="53"/>
-      <c r="B17" s="53"/>
+    <row r="17" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="84"/>
+      <c r="B17" s="81"/>
       <c r="C17" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>183</v>
+        <v>49</v>
       </c>
       <c r="G17" s="8">
         <v>46100</v>
@@ -1925,123 +2197,139 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="53"/>
-      <c r="B18" s="53"/>
-      <c r="C18" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="E18" s="43" t="s">
-        <v>180</v>
-      </c>
-      <c r="F18" s="21" t="s">
-        <v>54</v>
+    <row r="18" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="84"/>
+      <c r="B18" s="81"/>
+      <c r="C18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>179</v>
       </c>
       <c r="G18" s="8">
         <v>46100</v>
       </c>
       <c r="H18" s="9">
-        <v>46101</v>
-      </c>
-      <c r="I18" s="10">
-        <f>H18-G18</f>
-        <v>1</v>
+        <v>46116</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="J18" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="53"/>
-      <c r="B19" s="53"/>
+    <row r="19" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="84"/>
+      <c r="B19" s="81"/>
       <c r="C19" s="18" t="s">
         <v>51</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="E19" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" s="40" t="s">
+        <v>176</v>
+      </c>
+      <c r="F19" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="F19" s="21" t="s">
-        <v>54</v>
-      </c>
       <c r="G19" s="8">
         <v>46100</v>
       </c>
       <c r="H19" s="9">
-        <v>46106</v>
+        <v>46101</v>
       </c>
       <c r="I19" s="10">
         <f>H19-G19</f>
-        <v>6</v>
-      </c>
-      <c r="J19" s="11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="53"/>
-      <c r="B20" s="53"/>
+        <v>1</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="84"/>
+      <c r="B20" s="81"/>
       <c r="C20" s="18" t="s">
         <v>51</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>56</v>
+        <v>190</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>57</v>
+        <v>189</v>
       </c>
       <c r="F20" s="21" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="G20" s="8">
         <v>46100</v>
       </c>
       <c r="H20" s="9">
-        <v>46106</v>
+        <v>46115</v>
       </c>
       <c r="I20" s="10">
         <f>H20-G20</f>
-        <v>6</v>
-      </c>
-      <c r="J20" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="K20" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="85"/>
+      <c r="B21" s="82"/>
+      <c r="C21" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="G21" s="8">
+        <v>46111</v>
+      </c>
+      <c r="H21" s="9"/>
+      <c r="I21" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J21" s="11" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="17"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="17"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="17"/>
-    </row>
-    <row r="22" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="44" t="s">
-        <v>59</v>
-      </c>
-      <c r="B22" s="45" t="s">
-        <v>60</v>
+    <row r="22" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="66" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="69" t="s">
+        <v>58</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G22" s="8">
         <v>46100</v>
@@ -2056,20 +2344,20 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="44"/>
-      <c r="B23" s="44"/>
+    <row r="23" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="67"/>
+      <c r="B23" s="70"/>
       <c r="C23" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G23" s="8">
         <v>46100</v>
@@ -2085,17 +2373,17 @@
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="44"/>
-      <c r="B24" s="44"/>
+    <row r="24" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="67"/>
+      <c r="B24" s="70"/>
       <c r="C24" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F24" s="5" t="s">
         <v>40</v>
@@ -2113,17 +2401,17 @@
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="44"/>
-      <c r="B25" s="44"/>
+    <row r="25" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="67"/>
+      <c r="B25" s="70"/>
       <c r="C25" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F25" s="5" t="s">
         <v>40</v>
@@ -2141,17 +2429,17 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="44"/>
-      <c r="B26" s="44"/>
+    <row r="26" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="67"/>
+      <c r="B26" s="70"/>
       <c r="C26" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>40</v>
@@ -2169,17 +2457,17 @@
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="44"/>
-      <c r="B27" s="44"/>
+    <row r="27" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="67"/>
+      <c r="B27" s="70"/>
       <c r="C27" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F27" s="5" t="s">
         <v>40</v>
@@ -2197,20 +2485,20 @@
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="44"/>
-      <c r="B28" s="44"/>
+    <row r="28" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="67"/>
+      <c r="B28" s="70"/>
       <c r="C28" s="18" t="s">
         <v>51</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E28" s="20" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="F28" s="21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G28" s="8">
         <v>46100</v>
@@ -2226,110 +2514,143 @@
         <v>17</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="44"/>
-      <c r="B29" s="44"/>
+    <row r="29" spans="1:11" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="67"/>
+      <c r="B29" s="70"/>
       <c r="C29" s="18" t="s">
         <v>51</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E29" s="20" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F29" s="21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G29" s="8">
         <v>46100</v>
       </c>
       <c r="H29" s="9">
-        <v>46110</v>
+        <v>46115</v>
       </c>
       <c r="I29" s="10">
         <f>H29-G29</f>
-        <v>10</v>
-      </c>
-      <c r="J29" s="11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="17"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="17"/>
-      <c r="H30" s="17"/>
-      <c r="I30" s="17"/>
-      <c r="J30" s="17"/>
-    </row>
-    <row r="31" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="J29" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="67"/>
+      <c r="B30" s="70"/>
+      <c r="C30" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="D30" s="46" t="s">
+        <v>194</v>
+      </c>
+      <c r="E30" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F30" s="48" t="s">
+        <v>53</v>
+      </c>
+      <c r="G30" s="49">
+        <v>46101</v>
+      </c>
+      <c r="H30" s="50">
+        <v>46102</v>
+      </c>
+      <c r="I30" s="51">
+        <f>H30-G30</f>
+        <v>1</v>
+      </c>
+      <c r="J30" s="52" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="68"/>
+      <c r="B31" s="71"/>
+      <c r="C31" s="86"/>
+      <c r="D31" s="46" t="s">
+        <v>198</v>
+      </c>
+      <c r="E31" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="F31" s="48"/>
+      <c r="G31" s="49">
+        <v>46115</v>
+      </c>
+      <c r="H31" s="50">
+        <v>46117</v>
+      </c>
+      <c r="I31" s="51">
+        <f>H31-G31</f>
+        <v>2</v>
+      </c>
+      <c r="J31" s="12" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="43">
+        <v>4</v>
+      </c>
+      <c r="B32" s="44" t="s">
+        <v>74</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D32" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="E32" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="F32" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="G32" s="8">
+        <v>46100</v>
+      </c>
+      <c r="H32" s="9">
+        <v>46115</v>
+      </c>
+      <c r="I32" s="10">
+        <f>H32-G32</f>
+        <v>15</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="K32" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="64" t="s">
         <v>75</v>
       </c>
-      <c r="B31" s="23" t="s">
+      <c r="B33" s="62" t="s">
         <v>76</v>
       </c>
-      <c r="C31" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="D31" s="41" t="s">
+      <c r="C33" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="E31" s="20" t="s">
+      <c r="D33" s="23" t="s">
+        <v>175</v>
+      </c>
+      <c r="E33" s="39" t="s">
+        <v>184</v>
+      </c>
+      <c r="F33" s="25" t="s">
         <v>78</v>
-      </c>
-      <c r="F31" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="G31" s="8">
-        <v>46100</v>
-      </c>
-      <c r="H31" s="9">
-        <v>46106</v>
-      </c>
-      <c r="I31" s="10">
-        <f>H31-G31</f>
-        <v>6</v>
-      </c>
-      <c r="J31" s="11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="17"/>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="17"/>
-      <c r="I32" s="17"/>
-      <c r="J32" s="17"/>
-    </row>
-    <row r="33" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="46" t="s">
-        <v>79</v>
-      </c>
-      <c r="B33" s="47" t="s">
-        <v>80</v>
-      </c>
-      <c r="C33" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="D33" s="25" t="s">
-        <v>179</v>
-      </c>
-      <c r="E33" s="42" t="s">
-        <v>188</v>
-      </c>
-      <c r="F33" s="27" t="s">
-        <v>82</v>
       </c>
       <c r="G33" s="8">
         <v>46100</v>
@@ -2346,19 +2667,19 @@
       </c>
     </row>
     <row r="34" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="46"/>
-      <c r="B34" s="46"/>
-      <c r="C34" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="D34" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="E34" s="42" t="s">
-        <v>187</v>
-      </c>
-      <c r="F34" s="27" t="s">
-        <v>82</v>
+      <c r="A34" s="64"/>
+      <c r="B34" s="62"/>
+      <c r="C34" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="E34" s="39" t="s">
+        <v>183</v>
+      </c>
+      <c r="F34" s="25" t="s">
+        <v>78</v>
       </c>
       <c r="G34" s="8">
         <v>46100</v>
@@ -2375,19 +2696,19 @@
       </c>
     </row>
     <row r="35" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="46"/>
-      <c r="B35" s="46"/>
-      <c r="C35" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="D35" s="25" t="s">
-        <v>84</v>
-      </c>
-      <c r="E35" s="42" t="s">
-        <v>187</v>
-      </c>
-      <c r="F35" s="27" t="s">
-        <v>82</v>
+      <c r="A35" s="64"/>
+      <c r="B35" s="62"/>
+      <c r="C35" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="D35" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="E35" s="39" t="s">
+        <v>183</v>
+      </c>
+      <c r="F35" s="25" t="s">
+        <v>78</v>
       </c>
       <c r="G35" s="8">
         <v>46100</v>
@@ -2404,19 +2725,19 @@
       </c>
     </row>
     <row r="36" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="46"/>
-      <c r="B36" s="46"/>
-      <c r="C36" s="24" t="s">
+      <c r="A36" s="64"/>
+      <c r="B36" s="62"/>
+      <c r="C36" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="D36" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="D36" s="25" t="s">
-        <v>85</v>
-      </c>
-      <c r="E36" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="F36" s="27" t="s">
+      <c r="E36" s="24" t="s">
         <v>82</v>
+      </c>
+      <c r="F36" s="25" t="s">
+        <v>78</v>
       </c>
       <c r="G36" s="8">
         <v>46100</v>
@@ -2432,10 +2753,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="17"/>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
+    <row r="37" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="65"/>
+      <c r="B37" s="63"/>
+      <c r="C37" s="22" t="s">
+        <v>77</v>
+      </c>
       <c r="D37" s="17"/>
       <c r="E37" s="17"/>
       <c r="F37" s="17"/>
@@ -2444,33 +2767,84 @@
       <c r="I37" s="17"/>
       <c r="J37" s="17"/>
     </row>
-    <row r="39" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="48" t="s">
-        <v>87</v>
-      </c>
-      <c r="B39" s="48"/>
-      <c r="C39" s="48"/>
-      <c r="D39" s="48"/>
-      <c r="E39" s="48"/>
-      <c r="F39" s="48"/>
-      <c r="G39" s="48"/>
-      <c r="H39" s="48"/>
-      <c r="I39" s="48"/>
-      <c r="J39" s="48"/>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="61" t="s">
+        <v>83</v>
+      </c>
+      <c r="B38" s="61"/>
+      <c r="C38" s="61"/>
+      <c r="D38" s="61"/>
+      <c r="E38" s="61"/>
+      <c r="F38" s="61"/>
+      <c r="G38" s="61"/>
+      <c r="H38" s="61"/>
+      <c r="I38" s="61"/>
+      <c r="J38" s="61"/>
+    </row>
+    <row r="39" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C47" s="53"/>
+      <c r="D47" s="59"/>
+      <c r="E47" s="54"/>
+      <c r="F47" s="55"/>
+      <c r="G47" s="56"/>
+      <c r="H47" s="57"/>
+      <c r="I47" s="58"/>
+      <c r="J47" s="60"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="42"/>
+      <c r="B49" s="42"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="42"/>
+      <c r="B50" s="42"/>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="42"/>
+      <c r="B51" s="42"/>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="42"/>
+      <c r="B52" s="42"/>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="42"/>
+      <c r="B53" s="42"/>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="42"/>
+      <c r="B54" s="42"/>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="42"/>
+      <c r="B55" s="42"/>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" s="42"/>
+      <c r="B56" s="42"/>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="42"/>
+      <c r="B57" s="42"/>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="42"/>
+      <c r="B58" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A4:A10"/>
-    <mergeCell ref="B4:B10"/>
-    <mergeCell ref="A12:A20"/>
-    <mergeCell ref="B12:B20"/>
-    <mergeCell ref="A22:A29"/>
-    <mergeCell ref="B22:B29"/>
-    <mergeCell ref="A33:A36"/>
-    <mergeCell ref="B33:B36"/>
-    <mergeCell ref="A39:J39"/>
+    <mergeCell ref="B4:B12"/>
+    <mergeCell ref="A4:A12"/>
+    <mergeCell ref="B13:B21"/>
+    <mergeCell ref="A13:A21"/>
+    <mergeCell ref="A38:J38"/>
+    <mergeCell ref="B33:B37"/>
+    <mergeCell ref="A33:A37"/>
+    <mergeCell ref="A22:A31"/>
+    <mergeCell ref="B22:B31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2490,412 +2864,412 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="72" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+    </row>
+    <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="73" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+    </row>
+    <row r="3" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-    </row>
-    <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
+    </row>
+    <row r="4" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="28" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-    </row>
-    <row r="3" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="28" t="s">
+      <c r="C4" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="D4" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="D3" s="28" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" s="28" t="s">
+    </row>
+    <row r="5" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="29" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="29" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="30" t="s">
+      <c r="D5" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="C4" s="31" t="s">
+    </row>
+    <row r="6" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="27" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="D4" s="31" t="s">
+      <c r="C6" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="29" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="D7" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="31" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="31" t="s">
+      <c r="E7" s="29" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>101</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="29" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="29" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" s="29" t="s">
         <v>96</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="E10" s="29" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="31" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="B6" s="30" t="s">
-        <v>98</v>
-      </c>
-      <c r="C6" s="31" t="s">
-        <v>99</v>
-      </c>
-      <c r="D6" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="E6" s="31" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="29" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="C7" s="31" t="s">
-        <v>103</v>
-      </c>
-      <c r="D7" s="31" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="31" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="29" t="s">
-        <v>79</v>
-      </c>
-      <c r="B8" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="C8" s="31" t="s">
+      <c r="E11" s="29" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="B12" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="C12" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="31" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="31" t="s">
+      <c r="D12" s="29" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="29" t="s">
-        <v>108</v>
-      </c>
-      <c r="B9" s="30" t="s">
-        <v>109</v>
-      </c>
-      <c r="C9" s="31" t="s">
-        <v>110</v>
-      </c>
-      <c r="D9" s="31" t="s">
-        <v>111</v>
-      </c>
-      <c r="E9" s="31" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="29" t="s">
-        <v>113</v>
-      </c>
-      <c r="B10" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="C10" s="31" t="s">
-        <v>110</v>
-      </c>
-      <c r="D10" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="E10" s="31" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="29" t="s">
-        <v>116</v>
-      </c>
-      <c r="B11" s="30" t="s">
+      <c r="E12" s="29" t="s">
         <v>117</v>
       </c>
-      <c r="C11" s="31" t="s">
-        <v>110</v>
-      </c>
-      <c r="D11" s="31" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="31" t="s">
+    </row>
+    <row r="13" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="27" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="29" t="s">
+      <c r="B13" s="28" t="s">
         <v>119</v>
       </c>
-      <c r="B12" s="30" t="s">
+      <c r="C13" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="C12" s="31" t="s">
-        <v>110</v>
-      </c>
-      <c r="D12" s="31" t="s">
-        <v>111</v>
-      </c>
-      <c r="E12" s="31" t="s">
+      <c r="D13" s="29" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="29" t="s">
+      <c r="E13" s="29" t="s">
         <v>122</v>
       </c>
-      <c r="B13" s="30" t="s">
+    </row>
+    <row r="14" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="30" t="s">
         <v>123</v>
       </c>
-      <c r="C13" s="31" t="s">
+      <c r="B14" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="D13" s="31" t="s">
+      <c r="C14" s="32" t="s">
         <v>125</v>
       </c>
-      <c r="E13" s="31" t="s">
+      <c r="D14" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="E14" s="32" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="32" t="s">
+    <row r="15" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="30" t="s">
         <v>127</v>
       </c>
-      <c r="B14" s="33" t="s">
+      <c r="B15" s="31" t="s">
         <v>128</v>
       </c>
-      <c r="C14" s="34" t="s">
+      <c r="C15" s="32" t="s">
         <v>129</v>
       </c>
-      <c r="D14" s="34" t="s">
+      <c r="D15" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="34" t="s">
+      <c r="E15" s="32" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="32" t="s">
+    <row r="16" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="30" t="s">
         <v>131</v>
       </c>
-      <c r="B15" s="33" t="s">
+      <c r="B16" s="31" t="s">
         <v>132</v>
       </c>
-      <c r="C15" s="34" t="s">
+      <c r="C16" s="32" t="s">
         <v>133</v>
       </c>
-      <c r="D15" s="34" t="s">
+      <c r="D16" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="34" t="s">
+      <c r="E16" s="32" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="32" t="s">
+    <row r="17" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="30" t="s">
         <v>135</v>
       </c>
-      <c r="B16" s="33" t="s">
+      <c r="B17" s="31" t="s">
         <v>136</v>
       </c>
-      <c r="C16" s="34" t="s">
+      <c r="C17" s="32" t="s">
         <v>137</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="D17" s="32" t="s">
+        <v>138</v>
+      </c>
+      <c r="E17" s="32" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="30" t="s">
+        <v>140</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="C18" s="32" t="s">
+        <v>142</v>
+      </c>
+      <c r="D18" s="32" t="s">
+        <v>143</v>
+      </c>
+      <c r="E18" s="32" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="B19" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="C19" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="D19" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="E19" s="32" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B20" s="31" t="s">
+        <v>151</v>
+      </c>
+      <c r="C20" s="32" t="s">
+        <v>152</v>
+      </c>
+      <c r="D20" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="E20" s="32" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="B21" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="C21" s="32" t="s">
+        <v>156</v>
+      </c>
+      <c r="D21" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="E16" s="34" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="32" t="s">
-        <v>139</v>
-      </c>
-      <c r="B17" s="33" t="s">
-        <v>140</v>
-      </c>
-      <c r="C17" s="34" t="s">
-        <v>141</v>
-      </c>
-      <c r="D17" s="34" t="s">
-        <v>142</v>
-      </c>
-      <c r="E17" s="34" t="s">
+      <c r="E21" s="32" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B22" s="31" t="s">
+        <v>159</v>
+      </c>
+      <c r="C22" s="32" t="s">
+        <v>160</v>
+      </c>
+      <c r="D22" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="E22" s="32" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="B23" s="31" t="s">
+        <v>163</v>
+      </c>
+      <c r="C23" s="32" t="s">
+        <v>164</v>
+      </c>
+      <c r="D23" s="32" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="32" t="s">
-        <v>144</v>
-      </c>
-      <c r="B18" s="33" t="s">
-        <v>145</v>
-      </c>
-      <c r="C18" s="34" t="s">
-        <v>146</v>
-      </c>
-      <c r="D18" s="34" t="s">
-        <v>147</v>
-      </c>
-      <c r="E18" s="34" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="32" t="s">
-        <v>149</v>
-      </c>
-      <c r="B19" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="C19" s="34" t="s">
-        <v>151</v>
-      </c>
-      <c r="D19" s="34" t="s">
-        <v>152</v>
-      </c>
-      <c r="E19" s="34" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="32" t="s">
-        <v>154</v>
-      </c>
-      <c r="B20" s="33" t="s">
-        <v>155</v>
-      </c>
-      <c r="C20" s="34" t="s">
-        <v>156</v>
-      </c>
-      <c r="D20" s="34" t="s">
-        <v>152</v>
-      </c>
-      <c r="E20" s="34" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="32" t="s">
-        <v>158</v>
-      </c>
-      <c r="B21" s="33" t="s">
-        <v>159</v>
-      </c>
-      <c r="C21" s="34" t="s">
-        <v>160</v>
-      </c>
-      <c r="D21" s="34" t="s">
-        <v>51</v>
-      </c>
-      <c r="E21" s="34" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="B22" s="33" t="s">
-        <v>163</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>164</v>
-      </c>
-      <c r="D22" s="34" t="s">
-        <v>51</v>
-      </c>
-      <c r="E22" s="34" t="s">
+      <c r="E23" s="32" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="32" t="s">
+    <row r="24" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="33" t="s">
         <v>166</v>
       </c>
-      <c r="B23" s="33" t="s">
+      <c r="B24" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" s="35" t="s">
         <v>167</v>
       </c>
-      <c r="C23" s="34" t="s">
+      <c r="D24" s="35" t="s">
         <v>168</v>
       </c>
-      <c r="D23" s="34" t="s">
-        <v>147</v>
-      </c>
-      <c r="E23" s="34" t="s">
+      <c r="E24" s="35" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="35" t="s">
+    <row r="25" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="36" t="s">
         <v>170</v>
       </c>
-      <c r="B24" s="36" t="s">
-        <v>34</v>
-      </c>
-      <c r="C24" s="37" t="s">
+      <c r="B25" s="37" t="s">
         <v>171</v>
       </c>
-      <c r="D24" s="37" t="s">
+      <c r="C25" s="38" t="s">
         <v>172</v>
       </c>
-      <c r="E24" s="37" t="s">
+      <c r="D25" s="38" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="38" t="s">
+      <c r="E25" s="38" t="s">
         <v>174</v>
-      </c>
-      <c r="B25" s="39" t="s">
-        <v>175</v>
-      </c>
-      <c r="C25" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="D25" s="40" t="s">
-        <v>177</v>
-      </c>
-      <c r="E25" s="40" t="s">
-        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -2914,8 +3288,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
-        <v>191</v>
+      <c r="A1" s="41" t="s">
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>